<commit_message>
Planilha de bancos de bateria atualizada automaticamente
</commit_message>
<xml_diff>
--- a/dados/Controle de Bancos de Bateria Oficial.xlsx
+++ b/dados/Controle de Bancos de Bateria Oficial.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30431"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30502"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qinzen\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="751" documentId="13_ncr:1_{AD74628D-BE06-4FC1-BE04-2187DD70E9AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CCFE75F4-D69A-43D0-9A38-48CF2E5C2295}"/>
+  <xr:revisionPtr revIDLastSave="761" documentId="13_ncr:1_{AD74628D-BE06-4FC1-BE04-2187DD70E9AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A6EBADF6-010E-44D9-8F89-FE0D87C5128C}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13905" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1594" uniqueCount="573">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1657" uniqueCount="594">
   <si>
     <t>Id</t>
   </si>
@@ -1730,9 +1730,6 @@
     <t>Leandro</t>
   </si>
   <si>
-    <t>ECJ-FORQ-S07</t>
-  </si>
-  <si>
     <t>052920B</t>
   </si>
   <si>
@@ -1755,14 +1752,81 @@
   </si>
   <si>
     <t>015077A</t>
+  </si>
+  <si>
+    <t>0020745</t>
+  </si>
+  <si>
+    <t>sim</t>
+  </si>
+  <si>
+    <t>015084A</t>
+  </si>
+  <si>
+    <t>33/2025</t>
+  </si>
+  <si>
+    <t>4.35</t>
+  </si>
+  <si>
+    <t>015102A</t>
+  </si>
+  <si>
+    <t>12.06</t>
+  </si>
+  <si>
+    <t>4.29</t>
+  </si>
+  <si>
+    <t>052925B</t>
+  </si>
+  <si>
+    <t>29/2025</t>
+  </si>
+  <si>
+    <t>12.04</t>
+  </si>
+  <si>
+    <t>4.32</t>
+  </si>
+  <si>
+    <t>015069A</t>
+  </si>
+  <si>
+    <t>4.38</t>
+  </si>
+  <si>
+    <t>015171A</t>
+  </si>
+  <si>
+    <t>12.05</t>
+  </si>
+  <si>
+    <t>4.39</t>
+  </si>
+  <si>
+    <t>015078A</t>
+  </si>
+  <si>
+    <t>043016A</t>
+  </si>
+  <si>
+    <t>43/2025</t>
+  </si>
+  <si>
+    <t>052914B</t>
+  </si>
+  <si>
+    <t>https://icateltelematica.sharepoint.com/sites/Atividadessemanais-Planejamento/Shared%20Documents/LABORAT%C3%93RIO/Lista%20Baterias/Apps/Microsoft%20Forms/Controle%20de%20Bancos%20de%20Bateria%20Oficial/Relat%C3%B3rio/0020745_1x1s_Denilson%20de%20Oliveira.pdf</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -1810,7 +1874,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1878,6 +1942,17 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -2072,7 +2147,7 @@
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -2091,7 +2166,7 @@
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
       <alignment horizontal="left" vertical="center"/>
     </dxf>
     <dxf>
@@ -2131,8 +2206,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="OfficeForms.Table" displayName="OfficeForms.Table" ref="A1:BU40" totalsRowShown="0" headerRowDxfId="74" dataDxfId="73">
-  <autoFilter ref="A1:BU40" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="OfficeForms.Table" displayName="OfficeForms.Table" ref="A1:BU41" totalsRowShown="0" headerRowDxfId="74" dataDxfId="73">
+  <autoFilter ref="A1:BU41" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="73">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Id" dataDxfId="72">
       <extLst>
@@ -2631,7 +2706,7 @@
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
   <extLst>
     <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{839C7E11-91E4-4DBD-9C5D-0DEA604FA9AC}">
-      <xlmsforms:msForm id="KqFlZvtD4EW_4Nk20Gm35I7DWDUXhhxIi9Am8eUUGwZUOTNXUTJCRjZJRDVPVERQSzJJRzdZSVk5MCQlQCN0PWcu" isFormConnected="1" maxResponseId="40" latestEventMarker="59">
+      <xlmsforms:msForm id="KqFlZvtD4EW_4Nk20Gm35I7DWDUXhhxIi9Am8eUUGwZUOTNXUTJCRjZJRDVPVERQSzJJRzdZSVk5MCQlQCN0PWcu" isFormConnected="1" maxResponseId="41" latestEventMarker="60">
         <xlmsforms:syncedQuestionId>id</xlmsforms:syncedQuestionId>
         <xlmsforms:syncedQuestionId>startDate</xlmsforms:syncedQuestionId>
         <xlmsforms:syncedQuestionId>submitDate</xlmsforms:syncedQuestionId>
@@ -3005,7 +3080,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BU48"/>
+  <dimension ref="A1:BU49"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.42578125" customWidth="1"/>
@@ -9350,12 +9425,8 @@
         <v>563</v>
       </c>
       <c r="J40" s="1"/>
-      <c r="K40" s="14" t="s">
-        <v>564</v>
-      </c>
-      <c r="L40" s="2">
-        <v>46273</v>
-      </c>
+      <c r="K40" s="14"/>
+      <c r="L40" s="2"/>
       <c r="M40" s="1" t="s">
         <v>79</v>
       </c>
@@ -9363,7 +9434,7 @@
         <v>92</v>
       </c>
       <c r="O40" s="3" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="P40" s="19">
         <v>45858</v>
@@ -9380,7 +9451,7 @@
         <v>168</v>
       </c>
       <c r="V40" s="3" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="W40" s="15">
         <v>45870</v>
@@ -9397,7 +9468,7 @@
         <v>121</v>
       </c>
       <c r="AC40" s="3" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="AD40" s="15">
         <v>45870</v>
@@ -9414,7 +9485,7 @@
         <v>197</v>
       </c>
       <c r="AJ40" s="3" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="AK40" s="15">
         <v>45845</v>
@@ -9431,7 +9502,7 @@
         <v>168</v>
       </c>
       <c r="AQ40" s="1" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="AR40" s="15">
         <v>45870</v>
@@ -9448,7 +9519,7 @@
         <v>168</v>
       </c>
       <c r="AX40" s="1" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="AY40" s="15">
         <v>45870</v>
@@ -9465,7 +9536,7 @@
         <v>197</v>
       </c>
       <c r="BE40" s="1" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="BF40" s="15">
         <v>45839</v>
@@ -9482,7 +9553,7 @@
         <v>168</v>
       </c>
       <c r="BL40" s="1" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="BM40" s="30">
         <v>45870</v>
@@ -9503,14 +9574,223 @@
       <c r="BU40" s="1"/>
     </row>
     <row r="41" spans="1:73">
-      <c r="A41" s="5"/>
-      <c r="C41" s="23"/>
+      <c r="A41" s="1">
+        <v>41</v>
+      </c>
+      <c r="B41" s="23">
+        <v>46274.6402199074</v>
+      </c>
+      <c r="C41" s="23">
+        <v>46274.650543981501</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="F41" s="31"/>
+      <c r="G41" s="3" t="s">
+        <v>572</v>
+      </c>
+      <c r="H41" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="I41" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="J41" s="1"/>
+      <c r="K41" s="14"/>
+      <c r="L41" s="32"/>
+      <c r="M41" s="1" t="s">
+        <v>573</v>
+      </c>
+      <c r="N41" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="O41" s="3" t="s">
+        <v>574</v>
+      </c>
+      <c r="P41" s="33" t="s">
+        <v>575</v>
+      </c>
+      <c r="Q41" s="3" t="s">
+        <v>359</v>
+      </c>
+      <c r="R41" s="3" t="s">
+        <v>576</v>
+      </c>
+      <c r="S41" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="T41" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="U41" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="V41" s="3" t="s">
+        <v>577</v>
+      </c>
+      <c r="W41" s="34" t="s">
+        <v>575</v>
+      </c>
+      <c r="X41" s="3" t="s">
+        <v>578</v>
+      </c>
+      <c r="Y41" s="3" t="s">
+        <v>579</v>
+      </c>
+      <c r="Z41" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="AA41" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="AB41" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC41" s="3" t="s">
+        <v>580</v>
+      </c>
+      <c r="AD41" s="34" t="s">
+        <v>581</v>
+      </c>
+      <c r="AE41" s="3" t="s">
+        <v>582</v>
+      </c>
+      <c r="AF41" s="3" t="s">
+        <v>583</v>
+      </c>
+      <c r="AG41" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="AH41" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="AI41" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="AJ41" s="3" t="s">
+        <v>584</v>
+      </c>
+      <c r="AK41" s="34" t="s">
+        <v>575</v>
+      </c>
+      <c r="AL41" s="3" t="s">
+        <v>578</v>
+      </c>
+      <c r="AM41" s="3" t="s">
+        <v>585</v>
+      </c>
+      <c r="AN41" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="AO41" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="AP41" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="AQ41" s="1" t="s">
+        <v>586</v>
+      </c>
+      <c r="AR41" s="34" t="s">
+        <v>575</v>
+      </c>
+      <c r="AS41" s="3" t="s">
+        <v>587</v>
+      </c>
+      <c r="AT41" s="3" t="s">
+        <v>588</v>
+      </c>
+      <c r="AU41" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="AV41" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="AW41" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="AX41" s="1" t="s">
+        <v>589</v>
+      </c>
+      <c r="AY41" s="34" t="s">
+        <v>575</v>
+      </c>
+      <c r="AZ41" s="3" t="s">
+        <v>587</v>
+      </c>
+      <c r="BA41" s="3" t="s">
+        <v>585</v>
+      </c>
+      <c r="BB41" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="BC41" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="BD41" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="BE41" s="1" t="s">
+        <v>590</v>
+      </c>
+      <c r="BF41" s="34" t="s">
+        <v>591</v>
+      </c>
+      <c r="BG41" s="3" t="s">
+        <v>359</v>
+      </c>
+      <c r="BH41" s="3" t="s">
+        <v>588</v>
+      </c>
+      <c r="BI41" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="BJ41" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="BK41" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="BL41" s="1" t="s">
+        <v>592</v>
+      </c>
+      <c r="BM41" s="35" t="s">
+        <v>581</v>
+      </c>
+      <c r="BN41" s="3" t="s">
+        <v>578</v>
+      </c>
+      <c r="BO41" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="BP41" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="BQ41" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="BR41" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="BS41" s="10" t="s">
+        <v>593</v>
+      </c>
+      <c r="BT41" s="1"/>
+      <c r="BU41" s="1"/>
     </row>
-    <row r="45" spans="1:73">
-      <c r="R45" s="7"/>
+    <row r="42" spans="1:73">
+      <c r="A42" s="5"/>
+      <c r="C42" s="23"/>
     </row>
-    <row r="48" spans="1:73">
-      <c r="O48" s="7"/>
+    <row r="46" spans="1:73">
+      <c r="R46" s="7"/>
+    </row>
+    <row r="49" spans="15:15">
+      <c r="O49" s="7"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -9529,15 +9809,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="337ea2d0-885f-4217-baff-63e0aa38c74f">
@@ -9553,6 +9824,15 @@
     </Respons_x00e1_vel>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9783,11 +10063,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FC1EBE78-309B-4084-BAC4-28E69AD718B7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{360178F6-3CFF-461B-9986-D90DFFB5599F}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{360178F6-3CFF-461B-9986-D90DFFB5599F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FC1EBE78-309B-4084-BAC4-28E69AD718B7}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>